<commit_message>
feat: add 88th order (댕냥구리 구리본점)
</commit_message>
<xml_diff>
--- a/data/target_dispatch/파보겔_실제발송_최종정제명단.xlsx
+++ b/data/target_dispatch/파보겔_실제발송_최종정제명단.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="357">
   <si>
     <t>순번</t>
   </si>
@@ -298,6 +298,9 @@
     <t>디어마이펫</t>
   </si>
   <si>
+    <t>댕냥구리 강아지분양 고양이분양 구리본점</t>
+  </si>
+  <si>
     <t>정원정</t>
   </si>
   <si>
@@ -526,6 +529,9 @@
     <t>손명자</t>
   </si>
   <si>
+    <t>심우남</t>
+  </si>
+  <si>
     <t>010-3114-1100</t>
   </si>
   <si>
@@ -781,12 +787,15 @@
     <t>010-2982-6849</t>
   </si>
   <si>
-    <t>-</t>
+    <t>010-3848-5709</t>
   </si>
   <si>
     <t>010-8433-6449</t>
   </si>
   <si>
+    <t>010-7535-6488</t>
+  </si>
+  <si>
     <t>원주시 태장동 흥양로30  대흥아파트202-1202</t>
   </si>
   <si>
@@ -1046,6 +1055,9 @@
   </si>
   <si>
     <t>인천광역시 연수구 먼우금로 197, 114호</t>
+  </si>
+  <si>
+    <t>경기도 구리시 검배로6번길 8 댕냥구리</t>
   </si>
   <si>
     <t>[MMS 문자 유입] 펫샵 본품 1병 무료 샘플 신청</t>
@@ -1404,7 +1416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1438,19 +1450,19 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1461,19 +1473,19 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E3" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1484,19 +1496,19 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E4" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1507,19 +1519,19 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1530,19 +1542,19 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E6" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1553,19 +1565,19 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E7" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1576,19 +1588,19 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E8" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1599,19 +1611,19 @@
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E9" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1622,19 +1634,19 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E10" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1645,19 +1657,19 @@
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1668,19 +1680,19 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E12" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1691,19 +1703,19 @@
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D13" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E13" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1714,19 +1726,19 @@
         <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E14" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1737,19 +1749,19 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E15" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1760,19 +1772,19 @@
         <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D16" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E16" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1783,19 +1795,19 @@
         <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D17" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E17" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1806,19 +1818,19 @@
         <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D18" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E18" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
       <c r="G18" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1829,19 +1841,19 @@
         <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E19" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="G19" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1852,19 +1864,19 @@
         <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D20" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E20" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
       <c r="G20" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1875,19 +1887,19 @@
         <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E21" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1898,19 +1910,19 @@
         <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D22" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E22" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1921,19 +1933,19 @@
         <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D23" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E23" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="F23">
         <v>1</v>
       </c>
       <c r="G23" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1944,19 +1956,19 @@
         <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D24" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E24" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F24">
         <v>1</v>
       </c>
       <c r="G24" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1967,19 +1979,19 @@
         <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D25" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E25" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1990,19 +2002,19 @@
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D26" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E26" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2013,19 +2025,19 @@
         <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E27" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="G27" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2036,19 +2048,19 @@
         <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D28" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E28" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2059,19 +2071,19 @@
         <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D29" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E29" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F29">
         <v>1</v>
       </c>
       <c r="G29" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2082,19 +2094,19 @@
         <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E30" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2105,19 +2117,19 @@
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D31" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E31" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2128,19 +2140,19 @@
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D32" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E32" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F32">
         <v>1</v>
       </c>
       <c r="G32" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2151,19 +2163,19 @@
         <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D33" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E33" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="F33">
         <v>1</v>
       </c>
       <c r="G33" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2174,19 +2186,19 @@
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D34" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E34" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -2197,19 +2209,19 @@
         <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D35" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E35" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
       <c r="G35" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -2220,19 +2232,19 @@
         <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D36" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E36" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F36">
         <v>1</v>
       </c>
       <c r="G36" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2243,19 +2255,19 @@
         <v>42</v>
       </c>
       <c r="C37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D37" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E37" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -2266,19 +2278,19 @@
         <v>43</v>
       </c>
       <c r="C38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D38" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E38" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F38">
         <v>1</v>
       </c>
       <c r="G38" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -2289,19 +2301,19 @@
         <v>44</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D39" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E39" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F39">
         <v>1</v>
       </c>
       <c r="G39" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2312,19 +2324,19 @@
         <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D40" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E40" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F40">
         <v>1</v>
       </c>
       <c r="G40" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -2335,19 +2347,19 @@
         <v>46</v>
       </c>
       <c r="C41" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D41" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E41" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F41">
         <v>1</v>
       </c>
       <c r="G41" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -2358,19 +2370,19 @@
         <v>47</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D42" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E42" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F42">
         <v>1</v>
       </c>
       <c r="G42" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -2381,19 +2393,19 @@
         <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D43" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E43" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F43">
         <v>1</v>
       </c>
       <c r="G43" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -2404,19 +2416,19 @@
         <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D44" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E44" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F44">
         <v>1</v>
       </c>
       <c r="G44" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -2427,19 +2439,19 @@
         <v>50</v>
       </c>
       <c r="C45" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D45" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E45" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="F45">
         <v>1</v>
       </c>
       <c r="G45" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -2450,19 +2462,19 @@
         <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D46" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E46" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F46">
         <v>1</v>
       </c>
       <c r="G46" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -2473,19 +2485,19 @@
         <v>52</v>
       </c>
       <c r="C47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D47" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E47" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F47">
         <v>1</v>
       </c>
       <c r="G47" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2496,19 +2508,19 @@
         <v>53</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D48" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E48" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F48">
         <v>1</v>
       </c>
       <c r="G48" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -2519,19 +2531,19 @@
         <v>54</v>
       </c>
       <c r="C49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D49" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E49" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="F49">
         <v>1</v>
       </c>
       <c r="G49" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -2542,19 +2554,19 @@
         <v>55</v>
       </c>
       <c r="C50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D50" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E50" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F50">
         <v>1</v>
       </c>
       <c r="G50" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -2565,19 +2577,19 @@
         <v>56</v>
       </c>
       <c r="C51" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D51" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E51" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F51">
         <v>1</v>
       </c>
       <c r="G51" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -2588,19 +2600,19 @@
         <v>57</v>
       </c>
       <c r="C52" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D52" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E52" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F52">
         <v>1</v>
       </c>
       <c r="G52" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -2611,19 +2623,19 @@
         <v>58</v>
       </c>
       <c r="C53" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D53" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E53" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="F53">
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -2634,19 +2646,19 @@
         <v>59</v>
       </c>
       <c r="C54" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D54" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E54" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="F54">
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -2657,19 +2669,19 @@
         <v>60</v>
       </c>
       <c r="C55" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D55" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E55" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F55">
         <v>1</v>
       </c>
       <c r="G55" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -2680,19 +2692,19 @@
         <v>61</v>
       </c>
       <c r="C56" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D56" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E56" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F56">
         <v>1</v>
       </c>
       <c r="G56" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -2703,19 +2715,19 @@
         <v>62</v>
       </c>
       <c r="C57" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D57" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E57" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F57">
         <v>1</v>
       </c>
       <c r="G57" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -2726,19 +2738,19 @@
         <v>63</v>
       </c>
       <c r="C58" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D58" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E58" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F58">
         <v>1</v>
       </c>
       <c r="G58" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -2749,19 +2761,19 @@
         <v>64</v>
       </c>
       <c r="C59" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D59" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E59" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F59">
         <v>1</v>
       </c>
       <c r="G59" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -2772,19 +2784,19 @@
         <v>65</v>
       </c>
       <c r="C60" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D60" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E60" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F60">
         <v>1</v>
       </c>
       <c r="G60" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -2795,19 +2807,19 @@
         <v>66</v>
       </c>
       <c r="C61" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D61" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E61" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="F61">
         <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -2818,19 +2830,19 @@
         <v>67</v>
       </c>
       <c r="C62" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D62" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E62" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F62">
         <v>1</v>
       </c>
       <c r="G62" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -2841,19 +2853,19 @@
         <v>68</v>
       </c>
       <c r="C63" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D63" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E63" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F63">
         <v>1</v>
       </c>
       <c r="G63" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -2864,19 +2876,19 @@
         <v>69</v>
       </c>
       <c r="C64" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D64" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E64" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F64">
         <v>1</v>
       </c>
       <c r="G64" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -2887,19 +2899,19 @@
         <v>70</v>
       </c>
       <c r="C65" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D65" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E65" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F65">
         <v>3</v>
       </c>
       <c r="G65" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -2910,19 +2922,19 @@
         <v>71</v>
       </c>
       <c r="C66" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D66" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E66" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="F66">
         <v>1</v>
       </c>
       <c r="G66" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -2933,19 +2945,19 @@
         <v>72</v>
       </c>
       <c r="C67" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D67" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E67" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="F67">
         <v>1</v>
       </c>
       <c r="G67" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -2956,19 +2968,19 @@
         <v>73</v>
       </c>
       <c r="C68" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D68" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E68" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F68">
         <v>1</v>
       </c>
       <c r="G68" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -2979,19 +2991,19 @@
         <v>74</v>
       </c>
       <c r="C69" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D69" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E69" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F69">
         <v>1</v>
       </c>
       <c r="G69" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -3002,19 +3014,19 @@
         <v>75</v>
       </c>
       <c r="C70" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D70" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E70" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="F70">
         <v>1</v>
       </c>
       <c r="G70" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -3025,19 +3037,19 @@
         <v>76</v>
       </c>
       <c r="C71" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D71" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E71" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F71">
         <v>1</v>
       </c>
       <c r="G71" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3048,19 +3060,19 @@
         <v>77</v>
       </c>
       <c r="C72" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D72" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E72" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F72">
         <v>1</v>
       </c>
       <c r="G72" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3071,19 +3083,19 @@
         <v>78</v>
       </c>
       <c r="C73" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D73" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E73" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F73">
         <v>1</v>
       </c>
       <c r="G73" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -3094,19 +3106,19 @@
         <v>79</v>
       </c>
       <c r="C74" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D74" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E74" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F74">
         <v>1</v>
       </c>
       <c r="G74" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -3117,19 +3129,19 @@
         <v>80</v>
       </c>
       <c r="C75" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D75" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E75" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F75">
         <v>1</v>
       </c>
       <c r="G75" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -3140,19 +3152,19 @@
         <v>81</v>
       </c>
       <c r="C76" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D76" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E76" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F76">
         <v>1</v>
       </c>
       <c r="G76" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -3166,16 +3178,16 @@
         <v>82</v>
       </c>
       <c r="D77" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E77" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F77">
         <v>1</v>
       </c>
       <c r="G77" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -3189,16 +3201,16 @@
         <v>83</v>
       </c>
       <c r="D78" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E78" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F78">
         <v>1</v>
       </c>
       <c r="G78" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -3212,16 +3224,16 @@
         <v>84</v>
       </c>
       <c r="D79" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E79" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F79">
         <v>1</v>
       </c>
       <c r="G79" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -3235,16 +3247,16 @@
         <v>85</v>
       </c>
       <c r="D80" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E80" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F80">
         <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -3258,16 +3270,16 @@
         <v>86</v>
       </c>
       <c r="D81" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E81" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F81">
         <v>1</v>
       </c>
       <c r="G81" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -3281,16 +3293,16 @@
         <v>87</v>
       </c>
       <c r="D82" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E82" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F82">
         <v>1</v>
       </c>
       <c r="G82" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -3304,16 +3316,16 @@
         <v>88</v>
       </c>
       <c r="D83" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E83" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F83">
         <v>1</v>
       </c>
       <c r="G83" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -3327,16 +3339,16 @@
         <v>89</v>
       </c>
       <c r="D84" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E84" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="F84">
         <v>1</v>
       </c>
       <c r="G84" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -3350,16 +3362,16 @@
         <v>90</v>
       </c>
       <c r="D85" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E85" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="F85">
         <v>1</v>
       </c>
       <c r="G85" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -3370,19 +3382,19 @@
         <v>91</v>
       </c>
       <c r="C86" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D86" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E86" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F86">
         <v>1</v>
       </c>
       <c r="G86" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -3396,16 +3408,16 @@
         <v>92</v>
       </c>
       <c r="D87" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E87" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F87">
         <v>1</v>
       </c>
       <c r="G87" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -3419,16 +3431,39 @@
         <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E88" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="F88">
         <v>1</v>
       </c>
       <c r="G88" t="s">
-        <v>349</v>
+        <v>353</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>94</v>
+      </c>
+      <c r="C89" t="s">
+        <v>171</v>
+      </c>
+      <c r="D89" t="s">
+        <v>259</v>
+      </c>
+      <c r="E89" t="s">
+        <v>347</v>
+      </c>
+      <c r="F89">
+        <v>1</v>
+      </c>
+      <c r="G89" t="s">
+        <v>351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add 89th order (Parachiwo pom)
</commit_message>
<xml_diff>
--- a/data/target_dispatch/파보겔_실제발송_최종정제명단.xlsx
+++ b/data/target_dispatch/파보겔_실제발송_최종정제명단.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="361">
   <si>
     <t>순번</t>
   </si>
@@ -301,6 +301,9 @@
     <t>댕냥구리 강아지분양 고양이분양 구리본점</t>
   </si>
   <si>
+    <t>Parachiwo pom</t>
+  </si>
+  <si>
     <t>정원정</t>
   </si>
   <si>
@@ -532,6 +535,9 @@
     <t>심우남</t>
   </si>
   <si>
+    <t>유지혜</t>
+  </si>
+  <si>
     <t>010-3114-1100</t>
   </si>
   <si>
@@ -796,6 +802,9 @@
     <t>010-7535-6488</t>
   </si>
   <si>
+    <t>010-7575-1231</t>
+  </si>
+  <si>
     <t>원주시 태장동 흥양로30  대흥아파트202-1202</t>
   </si>
   <si>
@@ -1058,6 +1067,9 @@
   </si>
   <si>
     <t>경기도 구리시 검배로6번길 8 댕냥구리</t>
+  </si>
+  <si>
+    <t>전남 나주시 금천면 신가신촌길 9-11</t>
   </si>
   <si>
     <t>[MMS 문자 유입] 펫샵 본품 1병 무료 샘플 신청</t>
@@ -1416,7 +1428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1450,19 +1462,19 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1473,19 +1485,19 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E3" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1496,19 +1508,19 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E4" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1519,19 +1531,19 @@
         <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1542,19 +1554,19 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E6" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1565,19 +1577,19 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E7" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1588,19 +1600,19 @@
         <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E8" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1611,19 +1623,19 @@
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E9" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1634,19 +1646,19 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E10" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1657,19 +1669,19 @@
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E11" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1680,19 +1692,19 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1703,19 +1715,19 @@
         <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E13" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1726,19 +1738,19 @@
         <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E14" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1749,19 +1761,19 @@
         <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E15" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1772,19 +1784,19 @@
         <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D16" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E16" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1795,19 +1807,19 @@
         <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E17" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="G17" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1818,19 +1830,19 @@
         <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E18" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
       <c r="G18" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1841,19 +1853,19 @@
         <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E19" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
       <c r="G19" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1864,19 +1876,19 @@
         <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E20" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
       <c r="G20" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1887,19 +1899,19 @@
         <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E21" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1910,19 +1922,19 @@
         <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E22" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
       <c r="G22" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1933,19 +1945,19 @@
         <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D23" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E23" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F23">
         <v>1</v>
       </c>
       <c r="G23" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1956,19 +1968,19 @@
         <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E24" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F24">
         <v>1</v>
       </c>
       <c r="G24" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1979,19 +1991,19 @@
         <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D25" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E25" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2002,19 +2014,19 @@
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E26" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2025,19 +2037,19 @@
         <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D27" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E27" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="G27" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2048,19 +2060,19 @@
         <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E28" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2071,19 +2083,19 @@
         <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E29" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F29">
         <v>1</v>
       </c>
       <c r="G29" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2094,19 +2106,19 @@
         <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E30" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2117,19 +2129,19 @@
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E31" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2140,19 +2152,19 @@
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D32" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E32" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F32">
         <v>1</v>
       </c>
       <c r="G32" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2163,19 +2175,19 @@
         <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E33" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F33">
         <v>1</v>
       </c>
       <c r="G33" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2186,19 +2198,19 @@
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E34" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -2209,19 +2221,19 @@
         <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D35" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E35" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
       <c r="G35" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -2232,19 +2244,19 @@
         <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D36" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E36" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F36">
         <v>1</v>
       </c>
       <c r="G36" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2255,19 +2267,19 @@
         <v>42</v>
       </c>
       <c r="C37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E37" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -2278,19 +2290,19 @@
         <v>43</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D38" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E38" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="F38">
         <v>1</v>
       </c>
       <c r="G38" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -2301,19 +2313,19 @@
         <v>44</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D39" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E39" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F39">
         <v>1</v>
       </c>
       <c r="G39" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2324,19 +2336,19 @@
         <v>45</v>
       </c>
       <c r="C40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E40" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F40">
         <v>1</v>
       </c>
       <c r="G40" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -2347,19 +2359,19 @@
         <v>46</v>
       </c>
       <c r="C41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E41" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F41">
         <v>1</v>
       </c>
       <c r="G41" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -2370,19 +2382,19 @@
         <v>47</v>
       </c>
       <c r="C42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D42" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E42" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="F42">
         <v>1</v>
       </c>
       <c r="G42" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -2393,19 +2405,19 @@
         <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E43" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F43">
         <v>1</v>
       </c>
       <c r="G43" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -2416,19 +2428,19 @@
         <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D44" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E44" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F44">
         <v>1</v>
       </c>
       <c r="G44" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -2439,19 +2451,19 @@
         <v>50</v>
       </c>
       <c r="C45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D45" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E45" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F45">
         <v>1</v>
       </c>
       <c r="G45" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -2462,19 +2474,19 @@
         <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D46" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E46" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="F46">
         <v>1</v>
       </c>
       <c r="G46" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -2485,19 +2497,19 @@
         <v>52</v>
       </c>
       <c r="C47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E47" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F47">
         <v>1</v>
       </c>
       <c r="G47" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2508,19 +2520,19 @@
         <v>53</v>
       </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E48" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F48">
         <v>1</v>
       </c>
       <c r="G48" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -2531,19 +2543,19 @@
         <v>54</v>
       </c>
       <c r="C49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D49" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E49" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="F49">
         <v>1</v>
       </c>
       <c r="G49" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -2554,19 +2566,19 @@
         <v>55</v>
       </c>
       <c r="C50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D50" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E50" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="F50">
         <v>1</v>
       </c>
       <c r="G50" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -2577,19 +2589,19 @@
         <v>56</v>
       </c>
       <c r="C51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D51" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E51" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="F51">
         <v>1</v>
       </c>
       <c r="G51" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -2600,19 +2612,19 @@
         <v>57</v>
       </c>
       <c r="C52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D52" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E52" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F52">
         <v>1</v>
       </c>
       <c r="G52" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -2623,19 +2635,19 @@
         <v>58</v>
       </c>
       <c r="C53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D53" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E53" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F53">
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -2646,19 +2658,19 @@
         <v>59</v>
       </c>
       <c r="C54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D54" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E54" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F54">
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -2669,19 +2681,19 @@
         <v>60</v>
       </c>
       <c r="C55" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D55" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E55" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F55">
         <v>1</v>
       </c>
       <c r="G55" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -2692,19 +2704,19 @@
         <v>61</v>
       </c>
       <c r="C56" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D56" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E56" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F56">
         <v>1</v>
       </c>
       <c r="G56" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -2715,19 +2727,19 @@
         <v>62</v>
       </c>
       <c r="C57" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D57" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E57" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F57">
         <v>1</v>
       </c>
       <c r="G57" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -2738,19 +2750,19 @@
         <v>63</v>
       </c>
       <c r="C58" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D58" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E58" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="F58">
         <v>1</v>
       </c>
       <c r="G58" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -2761,19 +2773,19 @@
         <v>64</v>
       </c>
       <c r="C59" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D59" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="E59" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F59">
         <v>1</v>
       </c>
       <c r="G59" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -2784,19 +2796,19 @@
         <v>65</v>
       </c>
       <c r="C60" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D60" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E60" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F60">
         <v>1</v>
       </c>
       <c r="G60" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -2807,19 +2819,19 @@
         <v>66</v>
       </c>
       <c r="C61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D61" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E61" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F61">
         <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -2830,19 +2842,19 @@
         <v>67</v>
       </c>
       <c r="C62" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D62" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E62" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F62">
         <v>1</v>
       </c>
       <c r="G62" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -2853,19 +2865,19 @@
         <v>68</v>
       </c>
       <c r="C63" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D63" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E63" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="F63">
         <v>1</v>
       </c>
       <c r="G63" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -2876,19 +2888,19 @@
         <v>69</v>
       </c>
       <c r="C64" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D64" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E64" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="F64">
         <v>1</v>
       </c>
       <c r="G64" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -2899,19 +2911,19 @@
         <v>70</v>
       </c>
       <c r="C65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D65" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E65" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F65">
         <v>3</v>
       </c>
       <c r="G65" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -2922,19 +2934,19 @@
         <v>71</v>
       </c>
       <c r="C66" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D66" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E66" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F66">
         <v>1</v>
       </c>
       <c r="G66" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -2945,19 +2957,19 @@
         <v>72</v>
       </c>
       <c r="C67" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D67" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E67" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="F67">
         <v>1</v>
       </c>
       <c r="G67" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -2968,19 +2980,19 @@
         <v>73</v>
       </c>
       <c r="C68" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D68" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E68" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="F68">
         <v>1</v>
       </c>
       <c r="G68" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -2991,19 +3003,19 @@
         <v>74</v>
       </c>
       <c r="C69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D69" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E69" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F69">
         <v>1</v>
       </c>
       <c r="G69" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -3014,19 +3026,19 @@
         <v>75</v>
       </c>
       <c r="C70" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D70" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E70" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F70">
         <v>1</v>
       </c>
       <c r="G70" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -3037,19 +3049,19 @@
         <v>76</v>
       </c>
       <c r="C71" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D71" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E71" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F71">
         <v>1</v>
       </c>
       <c r="G71" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3060,19 +3072,19 @@
         <v>77</v>
       </c>
       <c r="C72" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D72" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E72" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="F72">
         <v>1</v>
       </c>
       <c r="G72" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3083,19 +3095,19 @@
         <v>78</v>
       </c>
       <c r="C73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D73" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E73" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F73">
         <v>1</v>
       </c>
       <c r="G73" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -3106,19 +3118,19 @@
         <v>79</v>
       </c>
       <c r="C74" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D74" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="E74" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="F74">
         <v>1</v>
       </c>
       <c r="G74" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -3129,19 +3141,19 @@
         <v>80</v>
       </c>
       <c r="C75" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D75" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E75" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F75">
         <v>1</v>
       </c>
       <c r="G75" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -3152,19 +3164,19 @@
         <v>81</v>
       </c>
       <c r="C76" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D76" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E76" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F76">
         <v>1</v>
       </c>
       <c r="G76" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -3178,16 +3190,16 @@
         <v>82</v>
       </c>
       <c r="D77" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E77" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F77">
         <v>1</v>
       </c>
       <c r="G77" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -3201,16 +3213,16 @@
         <v>83</v>
       </c>
       <c r="D78" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E78" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F78">
         <v>1</v>
       </c>
       <c r="G78" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -3224,16 +3236,16 @@
         <v>84</v>
       </c>
       <c r="D79" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E79" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F79">
         <v>1</v>
       </c>
       <c r="G79" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -3247,16 +3259,16 @@
         <v>85</v>
       </c>
       <c r="D80" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E80" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F80">
         <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -3270,16 +3282,16 @@
         <v>86</v>
       </c>
       <c r="D81" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E81" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="F81">
         <v>1</v>
       </c>
       <c r="G81" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -3293,16 +3305,16 @@
         <v>87</v>
       </c>
       <c r="D82" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E82" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="F82">
         <v>1</v>
       </c>
       <c r="G82" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -3316,16 +3328,16 @@
         <v>88</v>
       </c>
       <c r="D83" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E83" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F83">
         <v>1</v>
       </c>
       <c r="G83" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -3339,16 +3351,16 @@
         <v>89</v>
       </c>
       <c r="D84" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E84" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F84">
         <v>1</v>
       </c>
       <c r="G84" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -3362,16 +3374,16 @@
         <v>90</v>
       </c>
       <c r="D85" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E85" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="F85">
         <v>1</v>
       </c>
       <c r="G85" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -3382,19 +3394,19 @@
         <v>91</v>
       </c>
       <c r="C86" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D86" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E86" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F86">
         <v>1</v>
       </c>
       <c r="G86" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -3408,16 +3420,16 @@
         <v>92</v>
       </c>
       <c r="D87" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E87" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F87">
         <v>1</v>
       </c>
       <c r="G87" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -3431,16 +3443,16 @@
         <v>93</v>
       </c>
       <c r="D88" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E88" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="F88">
         <v>1</v>
       </c>
       <c r="G88" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -3451,19 +3463,42 @@
         <v>94</v>
       </c>
       <c r="C89" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D89" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="E89" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="F89">
         <v>1</v>
       </c>
       <c r="G89" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>95</v>
+      </c>
+      <c r="C90" t="s">
+        <v>173</v>
+      </c>
+      <c r="D90" t="s">
+        <v>262</v>
+      </c>
+      <c r="E90" t="s">
         <v>351</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+      <c r="G90" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>